<commit_message>
feat: mark PLC terminals and merge duplicate GND branches
</commit_message>
<xml_diff>
--- a/data/rules-source/ОЛ - Электродвигатель асинхронный_В2 [nsCQfC].xlsx
+++ b/data/rules-source/ОЛ - Электродвигатель асинхронный_В2 [nsCQfC].xlsx
@@ -26895,7 +26895,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7C12A1F-F7AA-4B2D-B809-F3DF97ECC2FF}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" customWidth="1"/>
@@ -26945,6 +26945,159 @@
       </c>
       <c r="C4" s="6" t="s">
         <v>676</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>im1-012</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>#Process Device Type</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Imd-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>im1-012</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>#Marking</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Imd-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>im1-012</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>#Device tag</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Imd-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>im1-013</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>#Process Device Type</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Imd-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>im1-013</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>#Marking</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Imd-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>im1-013</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>#Device tag</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Imd-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>im1-014</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>#Process Device Type</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Imd-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>im1-014</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>#Marking</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Imd-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>im1-014</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>#Device tag</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Imd-2</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>